<commit_message>
Refine work quantity statement modeling
</commit_message>
<xml_diff>
--- a/prepare-work-quantity-statement/assets/vor-template.xlsx
+++ b/prepare-work-quantity-statement/assets/vor-template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ВОР" sheetId="1" r:id="R341a2e04708340bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Расчётный реестр" sheetId="2" r:id="Re9f09c52b34f4904"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="3" r:id="R98408cb1c33a4957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Допущения" sheetId="4" r:id="R7be1b7e60ded4806"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения" sheetId="5" r:id="R6fc964d1e72144fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ВОР" sheetId="1" r:id="Rce2ee3dbff5b45fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Расчётный реестр" sheetId="2" r:id="R7ceb9a0a96b748c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="3" r:id="Rbb32b2b8aa0f4707"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Допущения" sheetId="4" r:id="R42c40f524525440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения" sheetId="5" r:id="Rda45b35c8b9a4100"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -523,7 +523,7 @@
         <x:v>№ п/п</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>Наименование работ</x:v>
+        <x:v>Наименование работ, ресурсов и затрат</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
         <x:v>Ед. изм.</x:v>
@@ -773,7 +773,7 @@
         <x:v>Зона / система</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
-        <x:v>Наименование работы</x:v>
+        <x:v>Наименование работы / связанного ресурса</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
         <x:v>Ед.</x:v>
@@ -813,6 +813,12 @@
       </x:c>
       <x:c r="Q5" s="11" t="str">
         <x:v>Статус</x:v>
+      </x:c>
+      <x:c r="R5" t="str">
+        <x:v>Тип строки</x:v>
+      </x:c>
+      <x:c r="S5" t="str">
+        <x:v>Родительский WORK-ID</x:v>
       </x:c>
     </x:row>
     <x:row r="6">

</xml_diff>